<commit_message>
g1-june26 water meter reading updated to avg apr-may since waterone readings were faulty
</commit_message>
<xml_diff>
--- a/db/wateron/avg-water-usage.xlsx
+++ b/db/wateron/avg-water-usage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\manapristine\db\wateron\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F57C13-EEE4-4970-9FFB-938379921ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5699478-DC8C-4EF5-8124-A6557C57CE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -773,14 +773,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M65"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -821,7 +821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -857,7 +857,7 @@
         <v>-0.61210626715674865</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -893,7 +893,7 @@
         <v>-0.79825275488930802</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -929,7 +929,7 @@
         <v>-0.59635702654599154</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -965,7 +965,7 @@
         <v>-0.70950461838844525</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>-0.83221618421330856</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>-0.6427201984887787</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>-0.38061041292639136</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>-0.9923444114203368</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>-0.66765140324963068</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>-0.74124652274869529</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>-0.57928317560912945</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>-0.51555638605998311</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>-0.75868178596739899</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>0.27385062693076512</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>-0.80196657207125976</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>-0.74607526355298803</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1411,14 +1411,15 @@
         <v>6751.5</v>
       </c>
       <c r="E18" s="2">
-        <v>11858</v>
+        <f>AVERAGE(C18:D18)</f>
+        <v>9304.75</v>
       </c>
       <c r="F18" s="2">
         <v>3271.5</v>
       </c>
       <c r="G18" s="2">
-        <f t="shared" si="2"/>
-        <v>10155.833333333334</v>
+        <f>(AVERAGE(C18:E18))</f>
+        <v>9304.75</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1426,14 +1427,14 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2">
         <f t="shared" si="0"/>
-        <v>8778.9666666666672</v>
+        <v>8098.1</v>
       </c>
       <c r="M18" s="3">
         <f t="shared" si="1"/>
-        <v>-0.62734794148134365</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-0.59601634951408355</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1469,7 +1470,7 @@
         <v>-0.67768583185292686</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1505,7 +1506,7 @@
         <v>-0.82768122085629503</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>-0.82247364779618248</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -1577,7 +1578,7 @@
         <v>-0.7927716350511077</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -1613,7 +1614,7 @@
         <v>-0.99979220635294441</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -1649,7 +1650,7 @@
         <v>-0.76958657906545924</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -1685,7 +1686,7 @@
         <v>-0.53019464789535187</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -1721,7 +1722,7 @@
         <v>-0.56491235691478969</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1757,7 +1758,7 @@
         <v>-0.29597641489847615</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>-0.83889510785707799</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>57</v>
       </c>
@@ -1829,7 +1830,7 @@
         <v>-0.54336126531539619</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1865,7 +1866,7 @@
         <v>-0.57096973256704409</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1901,7 +1902,7 @@
         <v>-0.54122058912478066</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1937,7 +1938,7 @@
         <v>-0.7975894143849076</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1973,7 +1974,7 @@
         <v>-0.42414736906848721</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -2009,7 +2010,7 @@
         <v>-0.99925235508149335</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -2045,7 +2046,7 @@
         <v>-0.99992851617043654</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -2081,7 +2082,7 @@
         <v>-0.62763549278373199</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>73</v>
       </c>
@@ -2117,7 +2118,7 @@
         <v>-0.51269809380871911</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -2153,7 +2154,7 @@
         <v>-0.35503346090088617</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -2189,7 +2190,7 @@
         <v>-0.90196884376669817</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>-0.70185481381710024</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>81</v>
       </c>
@@ -2261,7 +2262,7 @@
         <v>-0.66191560747434675</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -2297,7 +2298,7 @@
         <v>-0.99664678583244659</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>85</v>
       </c>
@@ -2333,7 +2334,7 @@
         <v>-0.97830802603036882</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -2369,7 +2370,7 @@
         <v>-0.55250467270417913</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -2405,7 +2406,7 @@
         <v>-0.2792905321009243</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -2441,7 +2442,7 @@
         <v>3.5048231511254015</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>92</v>
       </c>
@@ -2477,7 +2478,7 @@
         <v>-0.67101496178645226</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -2513,7 +2514,7 @@
         <v>-0.90596684122465831</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>96</v>
       </c>
@@ -2549,7 +2550,7 @@
         <v>-0.82152812716715851</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>98</v>
       </c>
@@ -2585,7 +2586,7 @@
         <v>-0.67420757991515856</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>100</v>
       </c>
@@ -2621,7 +2622,7 @@
         <v>-0.6234384502792093</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -2657,7 +2658,7 @@
         <v>-0.59489045467861046</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -2693,7 +2694,7 @@
         <v>-0.99731327243417522</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>106</v>
       </c>
@@ -2729,7 +2730,7 @@
         <v>-0.92764999328658038</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>108</v>
       </c>
@@ -2765,7 +2766,7 @@
         <v>-0.69463043456438156</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>110</v>
       </c>
@@ -2801,7 +2802,7 @@
         <v>-0.86118671747414266</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>112</v>
       </c>
@@ -2837,7 +2838,7 @@
         <v>-0.99923707939460438</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>114</v>
       </c>
@@ -2873,7 +2874,7 @@
         <v>-0.96892939575072501</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>116</v>
       </c>
@@ -2909,7 +2910,7 @@
         <v>-0.45165026939285641</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>117</v>
       </c>
@@ -2945,7 +2946,7 @@
         <v>-0.82159492190038774</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>119</v>
       </c>
@@ -2981,7 +2982,7 @@
         <v>-0.61014593467685885</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>121</v>
       </c>
@@ -3017,7 +3018,7 @@
         <v>-0.14921422506415694</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>123</v>
       </c>
@@ -3053,7 +3054,7 @@
         <v>-0.58193176357520426</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>125</v>
       </c>
@@ -3089,7 +3090,7 @@
         <v>-0.50491935969023616</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>127</v>
       </c>

</xml_diff>

<commit_message>
sep26 accounts updated with water meter updates
</commit_message>
<xml_diff>
--- a/db/wateron/avg-water-usage.xlsx
+++ b/db/wateron/avg-water-usage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\manapristine\db\wateron\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5699478-DC8C-4EF5-8124-A6557C57CE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65CFC72-2FB6-4180-9652-A97771017069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -844,17 +844,20 @@
         <f>(AVERAGE(C2:E2))</f>
         <v>4130.333333333333</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2">
+        <f>AVERAGE(C2:E2,G2)</f>
+        <v>4130.333333333333</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2">
         <f t="shared" ref="L2:L33" si="0">SUM(C2:K2)/COUNT(C2:K2)</f>
-        <v>3582.1666666666665</v>
+        <v>3673.5277777777774</v>
       </c>
       <c r="M2" s="3">
         <f t="shared" ref="M2:M33" si="1">IFERROR((F2-L2)/L2, 0)</f>
-        <v>-0.61210626715674865</v>
+        <v>-0.62175323447790876</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -880,17 +883,20 @@
         <f t="shared" ref="G3:G65" si="2">(AVERAGE(C3:E3))</f>
         <v>10069.333333333334</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2">
+        <f t="shared" ref="H3:H65" si="3">AVERAGE(C3:E3,G3)</f>
+        <v>10069.333333333334</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2">
         <f t="shared" si="0"/>
-        <v>8394.1666666666679</v>
+        <v>8673.3611111111113</v>
       </c>
       <c r="M3" s="3">
         <f t="shared" si="1"/>
-        <v>-0.79825275488930802</v>
+        <v>-0.80474697429229347</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -916,17 +922,20 @@
         <f t="shared" si="2"/>
         <v>10114.666666666666</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2">
+        <f t="shared" si="3"/>
+        <v>10114.666666666666</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2">
         <f t="shared" si="0"/>
-        <v>8802.3333333333321</v>
+        <v>9021.0555555555547</v>
       </c>
       <c r="M4" s="3">
         <f t="shared" si="1"/>
-        <v>-0.59635702654599154</v>
+        <v>-0.60614365158056149</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -952,17 +961,20 @@
         <f t="shared" si="2"/>
         <v>4703.5</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2">
+        <f t="shared" si="3"/>
+        <v>4703.5</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2">
         <f t="shared" si="0"/>
-        <v>3994.9</v>
+        <v>4113</v>
       </c>
       <c r="M5" s="3">
         <f t="shared" si="1"/>
-        <v>-0.70950461838844525</v>
+        <v>-0.71784585460734263</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -988,17 +1000,20 @@
         <f t="shared" si="2"/>
         <v>3808.8333333333335</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2">
+        <f t="shared" si="3"/>
+        <v>3808.8333333333335</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2">
         <f t="shared" si="0"/>
-        <v>3152.8666666666668</v>
+        <v>3262.1944444444448</v>
       </c>
       <c r="M6" s="3">
         <f t="shared" si="1"/>
-        <v>-0.83221618421330856</v>
+        <v>-0.83783921865819699</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1024,17 +1039,20 @@
         <f t="shared" si="2"/>
         <v>6861.166666666667</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2">
+        <f t="shared" si="3"/>
+        <v>6861.166666666667</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2">
         <f t="shared" si="0"/>
-        <v>5911.3333333333339</v>
+        <v>6069.6388888888896</v>
       </c>
       <c r="M7" s="3">
         <f t="shared" si="1"/>
-        <v>-0.6427201984887787</v>
+        <v>-0.65203860745879993</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1060,17 +1078,20 @@
         <f t="shared" si="2"/>
         <v>40.666666666666664</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2">
+        <f t="shared" si="3"/>
+        <v>40.666666666666664</v>
+      </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2">
         <f t="shared" si="0"/>
-        <v>37.133333333333333</v>
+        <v>37.722222222222221</v>
       </c>
       <c r="M8" s="3">
         <f t="shared" si="1"/>
-        <v>-0.38061041292639136</v>
+        <v>-0.39027982326951399</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1096,17 +1117,20 @@
         <f t="shared" si="2"/>
         <v>2771.5</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="2">
+        <f t="shared" si="3"/>
+        <v>2771.5</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2">
         <f t="shared" si="0"/>
-        <v>2220.6</v>
+        <v>2312.4166666666665</v>
       </c>
       <c r="M9" s="3">
         <f t="shared" si="1"/>
-        <v>-0.9923444114203368</v>
+        <v>-0.99264838372553965</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1132,17 +1156,20 @@
         <f t="shared" si="2"/>
         <v>2027.6666666666667</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <f t="shared" si="3"/>
+        <v>2027.6666666666667</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2">
         <f t="shared" si="0"/>
-        <v>1737.6333333333332</v>
+        <v>1785.9722222222219</v>
       </c>
       <c r="M10" s="3">
         <f t="shared" si="1"/>
-        <v>-0.66765140324963068</v>
+        <v>-0.67664670658682635</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1168,17 +1195,20 @@
         <f t="shared" si="2"/>
         <v>10311.5</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2">
+        <f t="shared" si="3"/>
+        <v>10311.5</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2">
         <f t="shared" si="0"/>
-        <v>8699.4</v>
+        <v>8968.0833333333339</v>
       </c>
       <c r="M11" s="3">
         <f t="shared" si="1"/>
-        <v>-0.74124652274869529</v>
+        <v>-0.74899876413577782</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -1204,17 +1234,20 @@
         <f t="shared" si="2"/>
         <v>891.16666666666663</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2">
+        <f t="shared" si="3"/>
+        <v>891.16666666666663</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2">
         <f t="shared" si="0"/>
-        <v>778.43333333333328</v>
+        <v>797.22222222222217</v>
       </c>
       <c r="M12" s="3">
         <f t="shared" si="1"/>
-        <v>-0.57928317560912945</v>
+        <v>-0.589198606271777</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1240,17 +1273,20 @@
         <f t="shared" si="2"/>
         <v>2416.5</v>
       </c>
-      <c r="H13" s="2"/>
+      <c r="H13" s="2">
+        <f t="shared" si="3"/>
+        <v>2416.5</v>
+      </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2">
         <f t="shared" si="0"/>
-        <v>2140.6</v>
+        <v>2186.5833333333335</v>
       </c>
       <c r="M13" s="3">
         <f t="shared" si="1"/>
-        <v>-0.51555638605998311</v>
+        <v>-0.52574412134608794</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
@@ -1276,17 +1312,20 @@
         <f t="shared" si="2"/>
         <v>2238.1666666666665</v>
       </c>
-      <c r="H14" s="2"/>
+      <c r="H14" s="2">
+        <f t="shared" si="3"/>
+        <v>2238.1666666666665</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2">
         <f t="shared" si="0"/>
-        <v>1881.3333333333333</v>
+        <v>1940.8055555555554</v>
       </c>
       <c r="M14" s="3">
         <f t="shared" si="1"/>
-        <v>-0.75868178596739899</v>
+        <v>-0.76607651462021786</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -1312,17 +1351,20 @@
         <f t="shared" si="2"/>
         <v>2050.5</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2">
+        <f t="shared" si="3"/>
+        <v>2050.5</v>
+      </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2">
         <f t="shared" si="0"/>
-        <v>2201.1999999999998</v>
+        <v>2176.0833333333335</v>
       </c>
       <c r="M15" s="3">
         <f t="shared" si="1"/>
-        <v>0.27385062693076512</v>
+        <v>0.28855359399532793</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -1348,17 +1390,20 @@
         <f t="shared" si="2"/>
         <v>4216.166666666667</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2">
+        <f t="shared" si="3"/>
+        <v>4216.166666666667</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2">
         <f t="shared" si="0"/>
-        <v>3512.0333333333338</v>
+        <v>3629.3888888888891</v>
       </c>
       <c r="M16" s="3">
         <f t="shared" si="1"/>
-        <v>-0.80196657207125976</v>
+        <v>-0.80836994290437636</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -1384,17 +1429,20 @@
         <f t="shared" si="2"/>
         <v>14541.5</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2">
+        <f t="shared" si="3"/>
+        <v>14541.5</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2">
         <f t="shared" si="0"/>
-        <v>12255.6</v>
+        <v>12636.583333333334</v>
       </c>
       <c r="M17" s="3">
         <f t="shared" si="1"/>
-        <v>-0.74607526355298803</v>
+        <v>-0.75373090036204404</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -1421,17 +1469,20 @@
         <f>(AVERAGE(C18:E18))</f>
         <v>9304.75</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2">
+        <f t="shared" si="3"/>
+        <v>9304.75</v>
+      </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2">
         <f t="shared" si="0"/>
-        <v>8098.1</v>
+        <v>8299.2083333333339</v>
       </c>
       <c r="M18" s="3">
         <f t="shared" si="1"/>
-        <v>-0.59601634951408355</v>
+        <v>-0.60580577464718022</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -1457,17 +1508,20 @@
         <f t="shared" si="2"/>
         <v>16303.333333333334</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2">
+        <f t="shared" si="3"/>
+        <v>16303.333333333334</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2">
         <f t="shared" si="0"/>
-        <v>13941.366666666665</v>
+        <v>14335.027777777776</v>
       </c>
       <c r="M19" s="3">
         <f t="shared" si="1"/>
-        <v>-0.67768583185292686</v>
+        <v>-0.68653705666578169</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -1493,17 +1547,20 @@
         <f t="shared" si="2"/>
         <v>11388.5</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2">
+        <f t="shared" si="3"/>
+        <v>11388.5</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2">
         <f t="shared" si="0"/>
-        <v>9436</v>
+        <v>9761.4166666666661</v>
       </c>
       <c r="M20" s="3">
         <f t="shared" si="1"/>
-        <v>-0.82768122085629503</v>
+        <v>-0.83342581763234502</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -1529,17 +1586,20 @@
         <f t="shared" si="2"/>
         <v>19748.833333333332</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2">
+        <f t="shared" si="3"/>
+        <v>19748.833333333332</v>
+      </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2">
         <f t="shared" si="0"/>
-        <v>16380.666666666666</v>
+        <v>16942.027777777777</v>
       </c>
       <c r="M21" s="3">
         <f t="shared" si="1"/>
-        <v>-0.82247364779618248</v>
+        <v>-0.82835584747332813</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -1565,17 +1625,20 @@
         <f t="shared" si="2"/>
         <v>10135.833333333334</v>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2">
+        <f t="shared" si="3"/>
+        <v>10135.833333333334</v>
+      </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2">
         <f t="shared" si="0"/>
-        <v>8459.2666666666664</v>
+        <v>8738.6944444444453</v>
       </c>
       <c r="M22" s="3">
         <f t="shared" si="1"/>
-        <v>-0.7927716350511077</v>
+        <v>-0.799397952274844</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -1601,17 +1664,20 @@
         <f t="shared" si="2"/>
         <v>6015.333333333333</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="2">
+        <f t="shared" si="3"/>
+        <v>6015.333333333333</v>
+      </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2">
         <f t="shared" si="0"/>
-        <v>4812.4666666666662</v>
+        <v>5012.9444444444443</v>
       </c>
       <c r="M23" s="3">
         <f t="shared" si="1"/>
-        <v>-0.99979220635294441</v>
+        <v>-0.99980051644077006</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -1637,17 +1703,20 @@
         <f t="shared" si="2"/>
         <v>3454.3333333333335</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2">
+        <f t="shared" si="3"/>
+        <v>3454.3333333333335</v>
+      </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2">
         <f t="shared" si="0"/>
-        <v>2896.9666666666667</v>
+        <v>2989.8611111111113</v>
       </c>
       <c r="M24" s="3">
         <f t="shared" si="1"/>
-        <v>-0.76958657906545924</v>
+        <v>-0.77674548241742924</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -1673,17 +1742,20 @@
         <f t="shared" si="2"/>
         <v>5298.666666666667</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="2">
+        <f t="shared" si="3"/>
+        <v>5298.666666666667</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2">
         <f t="shared" si="0"/>
-        <v>4678.5333333333338</v>
+        <v>4781.8888888888896</v>
       </c>
       <c r="M25" s="3">
         <f t="shared" si="1"/>
-        <v>-0.53019464789535187</v>
+        <v>-0.54034900202151648</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -1709,17 +1781,20 @@
         <f t="shared" si="2"/>
         <v>8756.8333333333339</v>
       </c>
-      <c r="H26" s="2"/>
+      <c r="H26" s="2">
+        <f t="shared" si="3"/>
+        <v>8756.8333333333339</v>
+      </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2">
         <f t="shared" si="0"/>
-        <v>7673.166666666667</v>
+        <v>7853.7777777777783</v>
       </c>
       <c r="M26" s="3">
         <f t="shared" si="1"/>
-        <v>-0.56491235691478969</v>
+        <v>-0.57491794465508461</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
@@ -1745,17 +1820,20 @@
         <f t="shared" si="2"/>
         <v>2586.5</v>
       </c>
-      <c r="H27" s="2"/>
+      <c r="H27" s="2">
+        <f t="shared" si="3"/>
+        <v>2586.5</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2">
         <f t="shared" si="0"/>
-        <v>2408.3000000000002</v>
+        <v>2438</v>
       </c>
       <c r="M27" s="3">
         <f t="shared" si="1"/>
-        <v>-0.29597641489847615</v>
+        <v>-0.30455291222313374</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -1781,17 +1859,20 @@
         <f t="shared" si="2"/>
         <v>1332.8333333333333</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2">
+        <f t="shared" si="3"/>
+        <v>1332.8333333333333</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2">
         <f t="shared" si="0"/>
-        <v>1101.7666666666667</v>
+        <v>1140.2777777777776</v>
       </c>
       <c r="M28" s="3">
         <f t="shared" si="1"/>
-        <v>-0.83889510785707799</v>
+        <v>-0.8443361753958587</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
@@ -1817,17 +1898,20 @@
         <f t="shared" si="2"/>
         <v>11164.666666666666</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2">
+        <f t="shared" si="3"/>
+        <v>11164.666666666666</v>
+      </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2">
         <f t="shared" si="0"/>
-        <v>9829.4333333333325</v>
+        <v>10051.972222222221</v>
       </c>
       <c r="M29" s="3">
         <f t="shared" si="1"/>
-        <v>-0.54336126531539619</v>
+        <v>-0.55347071193878472</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -1853,17 +1937,20 @@
         <f t="shared" si="2"/>
         <v>5123.333333333333</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="H30" s="2">
+        <f t="shared" si="3"/>
+        <v>5123.333333333333</v>
+      </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2">
         <f t="shared" si="0"/>
-        <v>4483.3666666666668</v>
+        <v>4590.0277777777774</v>
       </c>
       <c r="M30" s="3">
         <f t="shared" si="1"/>
-        <v>-0.57096973256704409</v>
+        <v>-0.5809393552447637</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -1889,17 +1976,20 @@
         <f t="shared" si="2"/>
         <v>11262</v>
       </c>
-      <c r="H31" s="2"/>
+      <c r="H31" s="2">
+        <f t="shared" si="3"/>
+        <v>11262</v>
+      </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2">
         <f t="shared" si="0"/>
-        <v>9919.7999999999993</v>
+        <v>10143.5</v>
       </c>
       <c r="M31" s="3">
         <f t="shared" si="1"/>
-        <v>-0.54122058912478066</v>
+        <v>-0.5513382954601469</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -1925,17 +2015,20 @@
         <f t="shared" si="2"/>
         <v>2441.3333333333335</v>
       </c>
-      <c r="H32" s="2"/>
+      <c r="H32" s="2">
+        <f t="shared" si="3"/>
+        <v>2441.3333333333335</v>
+      </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2">
         <f t="shared" si="0"/>
-        <v>2035.4666666666667</v>
+        <v>2103.1111111111113</v>
       </c>
       <c r="M32" s="3">
         <f t="shared" si="1"/>
-        <v>-0.7975894143849076</v>
+        <v>-0.80409974640743875</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -1961,17 +2054,20 @@
         <f t="shared" si="2"/>
         <v>3596.5</v>
       </c>
-      <c r="H33" s="2"/>
+      <c r="H33" s="2">
+        <f t="shared" si="3"/>
+        <v>3596.5</v>
+      </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2">
         <f t="shared" si="0"/>
-        <v>3251.7</v>
+        <v>3309.1666666666665</v>
       </c>
       <c r="M33" s="3">
         <f t="shared" si="1"/>
-        <v>-0.42414736906848721</v>
+        <v>-0.43414756988164188</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
@@ -1997,17 +2093,20 @@
         <f t="shared" si="2"/>
         <v>835.83333333333337</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2">
+        <f t="shared" si="3"/>
+        <v>835.83333333333337</v>
+      </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2">
-        <f t="shared" ref="L34:L65" si="3">SUM(C34:K34)/COUNT(C34:K34)</f>
-        <v>668.76666666666665</v>
+        <f t="shared" ref="L34:L65" si="4">SUM(C34:K34)/COUNT(C34:K34)</f>
+        <v>696.6111111111112</v>
       </c>
       <c r="M34" s="3">
-        <f t="shared" ref="M34:M65" si="4">IFERROR((F34-L34)/L34, 0)</f>
-        <v>-0.99925235508149335</v>
+        <f t="shared" ref="M34:M65" si="5">IFERROR((F34-L34)/L34, 0)</f>
+        <v>-0.99928223941303129</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -2033,17 +2132,20 @@
         <f t="shared" si="2"/>
         <v>26229.333333333332</v>
       </c>
-      <c r="H35" s="2"/>
+      <c r="H35" s="2">
+        <f t="shared" si="3"/>
+        <v>26229.333333333332</v>
+      </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2">
-        <f t="shared" si="3"/>
-        <v>20983.766666666666</v>
+        <f t="shared" si="4"/>
+        <v>21858.027777777777</v>
       </c>
       <c r="M35" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.99992851617043654</v>
+        <f t="shared" si="5"/>
+        <v>-0.99993137532739684</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
@@ -2069,17 +2171,20 @@
         <f t="shared" si="2"/>
         <v>9114.1666666666661</v>
       </c>
-      <c r="H36" s="2"/>
+      <c r="H36" s="2">
+        <f t="shared" si="3"/>
+        <v>9114.1666666666661</v>
+      </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2">
-        <f t="shared" si="3"/>
-        <v>7878.0333333333328</v>
+        <f t="shared" si="4"/>
+        <v>8084.0555555555547</v>
       </c>
       <c r="M36" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.62763549278373199</v>
+        <f t="shared" si="5"/>
+        <v>-0.63712520530811678</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
@@ -2105,17 +2210,20 @@
         <f t="shared" si="2"/>
         <v>9546.5</v>
       </c>
-      <c r="H37" s="2"/>
+      <c r="H37" s="2">
+        <f t="shared" si="3"/>
+        <v>9546.5</v>
+      </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2">
-        <f t="shared" si="3"/>
-        <v>8461.9</v>
+        <f t="shared" si="4"/>
+        <v>8642.6666666666661</v>
       </c>
       <c r="M37" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.51269809380871911</v>
+        <f t="shared" si="5"/>
+        <v>-0.52289031163221222</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
@@ -2141,17 +2249,20 @@
         <f t="shared" si="2"/>
         <v>1773.3333333333333</v>
       </c>
-      <c r="H38" s="2"/>
+      <c r="H38" s="2">
+        <f t="shared" si="3"/>
+        <v>1773.3333333333333</v>
+      </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2">
-        <f t="shared" si="3"/>
-        <v>1628.7666666666667</v>
+        <f t="shared" si="4"/>
+        <v>1652.8611111111111</v>
       </c>
       <c r="M38" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.35503346090088617</v>
+        <f t="shared" si="5"/>
+        <v>-0.36443540661815371</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
@@ -2177,17 +2288,20 @@
         <f t="shared" si="2"/>
         <v>993.83333333333337</v>
       </c>
-      <c r="H39" s="2"/>
+      <c r="H39" s="2">
+        <f t="shared" si="3"/>
+        <v>993.83333333333337</v>
+      </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2">
-        <f t="shared" si="3"/>
-        <v>810.9666666666667</v>
+        <f t="shared" si="4"/>
+        <v>841.44444444444446</v>
       </c>
       <c r="M39" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.90196884376669817</v>
+        <f t="shared" si="5"/>
+        <v>-0.90551960913772611</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
@@ -2213,17 +2327,20 @@
         <f t="shared" si="2"/>
         <v>4189</v>
       </c>
-      <c r="H40" s="2"/>
+      <c r="H40" s="2">
+        <f t="shared" si="3"/>
+        <v>4189</v>
+      </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2">
-        <f t="shared" si="3"/>
-        <v>3563.7</v>
+        <f t="shared" si="4"/>
+        <v>3667.9166666666665</v>
       </c>
       <c r="M40" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.70185481381710024</v>
+        <f t="shared" si="5"/>
+        <v>-0.71032602521867549</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
@@ -2249,17 +2366,20 @@
         <f t="shared" si="2"/>
         <v>9518</v>
       </c>
-      <c r="H41" s="2"/>
+      <c r="H41" s="2">
+        <f t="shared" si="3"/>
+        <v>9518</v>
+      </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
       <c r="L41" s="2">
-        <f t="shared" si="3"/>
-        <v>8166.6</v>
+        <f t="shared" si="4"/>
+        <v>8391.8333333333339</v>
       </c>
       <c r="M41" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.66191560747434675</v>
+        <f t="shared" si="5"/>
+        <v>-0.67098965263847787</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
@@ -2285,17 +2405,20 @@
         <f t="shared" si="2"/>
         <v>9313.1666666666661</v>
       </c>
-      <c r="H42" s="2"/>
+      <c r="H42" s="2">
+        <f t="shared" si="3"/>
+        <v>9313.1666666666661</v>
+      </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2">
-        <f t="shared" si="3"/>
-        <v>7455.5333333333328</v>
+        <f t="shared" si="4"/>
+        <v>7765.1388888888878</v>
       </c>
       <c r="M42" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.99664678583244659</v>
+        <f t="shared" si="5"/>
+        <v>-0.99678048256989038</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
@@ -2321,17 +2444,20 @@
         <f t="shared" si="2"/>
         <v>688.5</v>
       </c>
-      <c r="H43" s="2"/>
+      <c r="H43" s="2">
+        <f t="shared" si="3"/>
+        <v>688.5</v>
+      </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2">
-        <f t="shared" si="3"/>
-        <v>553.20000000000005</v>
+        <f t="shared" si="4"/>
+        <v>575.75</v>
       </c>
       <c r="M43" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.97830802603036882</v>
+        <f t="shared" si="5"/>
+        <v>-0.97915762049500654</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
@@ -2357,17 +2483,20 @@
         <f t="shared" si="2"/>
         <v>3673.8333333333335</v>
       </c>
-      <c r="H44" s="2"/>
+      <c r="H44" s="2">
+        <f t="shared" si="3"/>
+        <v>3673.8333333333335</v>
+      </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2">
-        <f t="shared" si="3"/>
-        <v>3227.9666666666667</v>
+        <f t="shared" si="4"/>
+        <v>3302.2777777777778</v>
       </c>
       <c r="M44" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.55250467270417913</v>
+        <f t="shared" si="5"/>
+        <v>-0.56257465385844785</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
@@ -2393,17 +2522,20 @@
         <f t="shared" si="2"/>
         <v>4282.5</v>
       </c>
-      <c r="H45" s="2"/>
+      <c r="H45" s="2">
+        <f t="shared" si="3"/>
+        <v>4282.5</v>
+      </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2">
-        <f t="shared" si="3"/>
-        <v>4003</v>
+        <f t="shared" si="4"/>
+        <v>4049.5833333333335</v>
       </c>
       <c r="M45" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.2792905321009243</v>
+        <f t="shared" si="5"/>
+        <v>-0.28758102685461467</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
@@ -2429,17 +2561,20 @@
         <f t="shared" si="2"/>
         <v>12.833333333333334</v>
       </c>
-      <c r="H46" s="2"/>
+      <c r="H46" s="2">
+        <f t="shared" si="3"/>
+        <v>12.833333333333334</v>
+      </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2">
-        <f t="shared" si="3"/>
-        <v>103.66666666666667</v>
+        <f t="shared" si="4"/>
+        <v>88.527777777777786</v>
       </c>
       <c r="M46" s="4">
-        <f t="shared" si="4"/>
-        <v>3.5048231511254015</v>
+        <f t="shared" si="5"/>
+        <v>4.2751804204581108</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
@@ -2465,17 +2600,20 @@
         <f t="shared" si="2"/>
         <v>6254.333333333333</v>
       </c>
-      <c r="H47" s="2"/>
+      <c r="H47" s="2">
+        <f t="shared" si="3"/>
+        <v>6254.333333333333</v>
+      </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="2">
-        <f t="shared" si="3"/>
-        <v>5355.8666666666668</v>
+        <f t="shared" si="4"/>
+        <v>5505.6111111111104</v>
       </c>
       <c r="M47" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.67101496178645226</v>
+        <f t="shared" si="5"/>
+        <v>-0.67996286616683987</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
@@ -2501,17 +2639,20 @@
         <f t="shared" si="2"/>
         <v>15051.833333333334</v>
       </c>
-      <c r="H48" s="2"/>
+      <c r="H48" s="2">
+        <f t="shared" si="3"/>
+        <v>15051.833333333334</v>
+      </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2">
-        <f t="shared" si="3"/>
-        <v>12272.266666666666</v>
+        <f t="shared" si="4"/>
+        <v>12735.527777777779</v>
       </c>
       <c r="M48" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.90596684122465831</v>
+        <f t="shared" si="5"/>
+        <v>-0.90938734380418729</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -2537,17 +2678,20 @@
         <f t="shared" si="2"/>
         <v>2954.8333333333335</v>
       </c>
-      <c r="H49" s="2"/>
+      <c r="H49" s="2">
+        <f t="shared" si="3"/>
+        <v>2954.8333333333335</v>
+      </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2">
-        <f t="shared" si="3"/>
-        <v>2451.3666666666668</v>
+        <f t="shared" si="4"/>
+        <v>2535.2777777777778</v>
       </c>
       <c r="M49" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.82152812716715851</v>
+        <f t="shared" si="5"/>
+        <v>-0.82743508272159527</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
@@ -2573,17 +2717,20 @@
         <f t="shared" si="2"/>
         <v>15912.833333333334</v>
       </c>
-      <c r="H50" s="2"/>
+      <c r="H50" s="2">
+        <f t="shared" si="3"/>
+        <v>15912.833333333334</v>
+      </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="2">
-        <f t="shared" si="3"/>
-        <v>13617.566666666666</v>
+        <f t="shared" si="4"/>
+        <v>14000.111111111109</v>
       </c>
       <c r="M50" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.67420757991515856</v>
+        <f t="shared" si="5"/>
+        <v>-0.68310965785985822</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
@@ -2609,17 +2756,20 @@
         <f t="shared" si="2"/>
         <v>13240.333333333334</v>
       </c>
-      <c r="H51" s="2"/>
+      <c r="H51" s="2">
+        <f t="shared" si="3"/>
+        <v>13240.333333333334</v>
+      </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
       <c r="L51" s="2">
-        <f t="shared" si="3"/>
-        <v>11454.966666666667</v>
+        <f t="shared" si="4"/>
+        <v>11752.527777777779</v>
       </c>
       <c r="M51" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.6234384502792093</v>
+        <f t="shared" si="5"/>
+        <v>-0.63297257563975606</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
@@ -2645,17 +2795,20 @@
         <f t="shared" si="2"/>
         <v>7450.5</v>
       </c>
-      <c r="H52" s="2"/>
+      <c r="H52" s="2">
+        <f t="shared" si="3"/>
+        <v>7450.5</v>
+      </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
       <c r="L52" s="2">
-        <f t="shared" si="3"/>
-        <v>6485.9</v>
+        <f t="shared" si="4"/>
+        <v>6646.666666666667</v>
       </c>
       <c r="M52" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.59489045467861046</v>
+        <f t="shared" si="5"/>
+        <v>-0.60468906720160487</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.25">
@@ -2681,17 +2834,20 @@
         <f t="shared" si="2"/>
         <v>232.5</v>
       </c>
-      <c r="H53" s="2"/>
+      <c r="H53" s="2">
+        <f t="shared" si="3"/>
+        <v>232.5</v>
+      </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
       <c r="L53" s="2">
-        <f t="shared" si="3"/>
-        <v>186.1</v>
+        <f t="shared" si="4"/>
+        <v>193.83333333333334</v>
       </c>
       <c r="M53" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.99731327243417522</v>
+        <f t="shared" si="5"/>
+        <v>-0.99742046431642306</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
@@ -2717,17 +2873,20 @@
         <f t="shared" si="2"/>
         <v>3975.8333333333335</v>
       </c>
-      <c r="H54" s="2"/>
+      <c r="H54" s="2">
+        <f t="shared" si="3"/>
+        <v>3975.8333333333335</v>
+      </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="2">
-        <f t="shared" si="3"/>
-        <v>3227.3666666666668</v>
+        <f t="shared" si="4"/>
+        <v>3352.1111111111113</v>
       </c>
       <c r="M54" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.92764999328658038</v>
+        <f t="shared" si="5"/>
+        <v>-0.93034240445490402</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
@@ -2753,17 +2912,20 @@
         <f t="shared" si="2"/>
         <v>15588.833333333334</v>
       </c>
-      <c r="H55" s="2"/>
+      <c r="H55" s="2">
+        <f t="shared" si="3"/>
+        <v>15588.833333333334</v>
+      </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2">
-        <f t="shared" si="3"/>
-        <v>13282.266666666666</v>
+        <f t="shared" si="4"/>
+        <v>13666.694444444443</v>
       </c>
       <c r="M55" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.69463043456438156</v>
+        <f t="shared" si="5"/>
+        <v>-0.7032201154062695</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
@@ -2789,17 +2951,20 @@
         <f t="shared" si="2"/>
         <v>13246.166666666666</v>
       </c>
-      <c r="H56" s="2"/>
+      <c r="H56" s="2">
+        <f t="shared" si="3"/>
+        <v>13246.166666666666</v>
+      </c>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2">
-        <f t="shared" si="3"/>
-        <v>10899.533333333333</v>
+        <f t="shared" si="4"/>
+        <v>11290.638888888889</v>
       </c>
       <c r="M56" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.86118671747414266</v>
+        <f t="shared" si="5"/>
+        <v>-0.86599518283336985</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
@@ -2825,17 +2990,20 @@
         <f t="shared" si="2"/>
         <v>5733.666666666667</v>
       </c>
-      <c r="H57" s="2"/>
+      <c r="H57" s="2">
+        <f t="shared" si="3"/>
+        <v>5733.666666666667</v>
+      </c>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
       <c r="L57" s="2">
-        <f t="shared" si="3"/>
-        <v>4587.6333333333332</v>
+        <f t="shared" si="4"/>
+        <v>4778.6388888888896</v>
       </c>
       <c r="M57" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.99923707939460438</v>
+        <f t="shared" si="5"/>
+        <v>-0.99926757386750065</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
@@ -2861,17 +3029,20 @@
         <f t="shared" si="2"/>
         <v>699.66666666666663</v>
       </c>
-      <c r="H58" s="2"/>
+      <c r="H58" s="2">
+        <f t="shared" si="3"/>
+        <v>699.66666666666663</v>
+      </c>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
       <c r="L58" s="2">
-        <f t="shared" si="3"/>
-        <v>563.23333333333335</v>
+        <f t="shared" si="4"/>
+        <v>585.97222222222217</v>
       </c>
       <c r="M58" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.96892939575072501</v>
+        <f t="shared" si="5"/>
+        <v>-0.97013510310500117</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
@@ -2897,17 +3068,20 @@
         <f t="shared" si="2"/>
         <v>9735.8333333333339</v>
       </c>
-      <c r="H59" s="2"/>
+      <c r="H59" s="2">
+        <f t="shared" si="3"/>
+        <v>9735.8333333333339</v>
+      </c>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
       <c r="L59" s="2">
-        <f t="shared" si="3"/>
-        <v>8748.0666666666675</v>
+        <f t="shared" si="4"/>
+        <v>8912.6944444444453</v>
       </c>
       <c r="M59" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.45165026939285641</v>
+        <f t="shared" si="5"/>
+        <v>-0.46177892332098103</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
@@ -2933,17 +3107,20 @@
         <f t="shared" si="2"/>
         <v>5564</v>
       </c>
-      <c r="H60" s="2"/>
+      <c r="H60" s="2">
+        <f t="shared" si="3"/>
+        <v>5564</v>
+      </c>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
       <c r="L60" s="2">
-        <f t="shared" si="3"/>
-        <v>4615.8999999999996</v>
+        <f t="shared" si="4"/>
+        <v>4773.916666666667</v>
       </c>
       <c r="M60" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.82159492190038774</v>
+        <f t="shared" si="5"/>
+        <v>-0.82750013091975494</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
@@ -2969,17 +3146,20 @@
         <f t="shared" si="2"/>
         <v>2764.1666666666665</v>
       </c>
-      <c r="H61" s="2"/>
+      <c r="H61" s="2">
+        <f t="shared" si="3"/>
+        <v>2764.1666666666665</v>
+      </c>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
       <c r="L61" s="2">
-        <f t="shared" si="3"/>
-        <v>2398.333333333333</v>
+        <f t="shared" si="4"/>
+        <v>2459.3055555555552</v>
       </c>
       <c r="M61" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.61014593467685885</v>
+        <f t="shared" si="5"/>
+        <v>-0.61981137403286835</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
@@ -3005,17 +3185,20 @@
         <f t="shared" si="2"/>
         <v>7289.166666666667</v>
       </c>
-      <c r="H62" s="2"/>
+      <c r="H62" s="2">
+        <f t="shared" si="3"/>
+        <v>7289.166666666667</v>
+      </c>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
       <c r="L62" s="2">
-        <f t="shared" si="3"/>
-        <v>7027.0333333333328</v>
+        <f t="shared" si="4"/>
+        <v>7070.7222222222217</v>
       </c>
       <c r="M62" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.14921422506415694</v>
+        <f t="shared" si="5"/>
+        <v>-0.15447109756193372</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
@@ -3041,17 +3224,20 @@
         <f t="shared" si="2"/>
         <v>6992.333333333333</v>
       </c>
-      <c r="H63" s="2"/>
+      <c r="H63" s="2">
+        <f t="shared" si="3"/>
+        <v>6992.333333333333</v>
+      </c>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
       <c r="L63" s="2">
-        <f t="shared" si="3"/>
-        <v>6104.2666666666664</v>
+        <f t="shared" si="4"/>
+        <v>6252.2777777777774</v>
       </c>
       <c r="M63" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.58193176357520426</v>
+        <f t="shared" si="5"/>
+        <v>-0.59182875574235161</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
@@ -3077,17 +3263,20 @@
         <f t="shared" si="2"/>
         <v>6864.333333333333</v>
       </c>
-      <c r="H64" s="2"/>
+      <c r="H64" s="2">
+        <f t="shared" si="3"/>
+        <v>6864.333333333333</v>
+      </c>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
       <c r="L64" s="2">
-        <f t="shared" si="3"/>
-        <v>6094.9666666666662</v>
+        <f t="shared" si="4"/>
+        <v>6223.1944444444443</v>
       </c>
       <c r="M64" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.50491935969023616</v>
+        <f t="shared" si="5"/>
+        <v>-0.51512040529381564</v>
       </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
@@ -3113,17 +3302,20 @@
         <f t="shared" si="2"/>
         <v>11086.5</v>
       </c>
-      <c r="H65" s="2"/>
+      <c r="H65" s="2">
+        <f t="shared" si="3"/>
+        <v>11086.5</v>
+      </c>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
       <c r="L65" s="2">
-        <f t="shared" si="3"/>
-        <v>9614.4</v>
+        <f t="shared" si="4"/>
+        <v>9859.75</v>
       </c>
       <c r="M65" s="3">
-        <f t="shared" si="4"/>
-        <v>-0.61245631552670987</v>
+        <f t="shared" si="5"/>
+        <v>-0.62209995182433631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>